<commit_message>
feat: done thiet bi do import
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
+++ b/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qcadoo_demo\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1ABB391-1E0F-4557-A31B-7C20A7FF19E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{055C28C7-E7B7-45A4-B8AA-485BA6188513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
   </bookViews>
@@ -36,15 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Measuring method</t>
   </si>
   <si>
     <t>Name</t>
-  </si>
-  <si>
-    <t>Number</t>
   </si>
 </sst>
 </file>
@@ -416,22 +413,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DC442A8-9B14-43DD-AF19-A2F9911D2500}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: an update of thiet bi do
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
+++ b/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qcadoo_demo\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{055C28C7-E7B7-45A4-B8AA-485BA6188513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCEAA18-FDC9-4461-AC9B-4BC4D4D4426B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
+    <workbookView xWindow="4545" yWindow="2715" windowWidth="21600" windowHeight="11235" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,8 +48,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -77,8 +85,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,10 +433,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
done thiet bi do
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
+++ b/src/main/resources/qm/public/resources/measuringEquipmentImportSchema_en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qcadoo_demo\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qcadoo_demo_clone\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCEAA18-FDC9-4461-AC9B-4BC4D4D4426B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF92491-5E7C-48C5-B3AC-BE8E51277A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4545" yWindow="2715" windowWidth="21600" windowHeight="11235" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
+    <workbookView xWindow="4890" yWindow="3060" windowWidth="21600" windowHeight="11235" xr2:uid="{68D7CCB2-5FFD-43FB-9C40-727480D7EABE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Measuring method</t>
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Equipment Code</t>
   </si>
 </sst>
 </file>
@@ -424,23 +427,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DC442A8-9B14-43DD-AF19-A2F9911D2500}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>